<commit_message>
Tried to avoid dependence on the bruges library in blixt_geo_py
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_geo_py\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F6DBF4-8BF0-4ACE-B5A2-16BA92B81AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9026C1CA-D41D-4D58-890B-D64555C54D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6570" yWindow="2745" windowWidth="28800" windowHeight="17145" tabRatio="685" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7170" yWindow="3090" windowWidth="28800" windowHeight="15345" tabRatio="685" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -682,9 +682,6 @@
     <t>Impedance</t>
   </si>
   <si>
-    <t>$MPa s/m$</t>
-  </si>
-  <si>
     <t>#8c564b</t>
   </si>
   <si>
@@ -710,9 +707,6 @@
   </si>
   <si>
     <t>SW,SW_RSI,SW_CPI</t>
-  </si>
-  <si>
-    <t>g/cm$^3$</t>
   </si>
   <si>
     <t>NEU</t>
@@ -1289,6 +1283,12 @@
   </si>
   <si>
     <t>Group B</t>
+  </si>
+  <si>
+    <t>MPa s/m</t>
+  </si>
+  <si>
+    <t>g/cm^3</t>
   </si>
 </sst>
 </file>
@@ -2193,7 +2193,7 @@
         <v>21</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2250,38 +2250,38 @@
   <sheetData>
     <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
+        <v>252</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>255</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="E2" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="F2" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="D2" s="34" t="s">
-        <v>257</v>
-      </c>
-      <c r="E2" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="F2" s="33" t="s">
-        <v>258</v>
-      </c>
       <c r="G2" s="33" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B3">
         <v>36.6</v>
@@ -2298,7 +2298,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B4">
         <v>11.4</v>
@@ -2313,15 +2313,15 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="G4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B5">
         <v>76.8</v>
@@ -2338,7 +2338,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B6">
         <v>94.9</v>
@@ -2355,7 +2355,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B7">
         <v>26</v>
@@ -2372,7 +2372,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B8">
         <v>47</v>
@@ -2389,7 +2389,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B9">
         <v>114</v>
@@ -2406,7 +2406,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B10">
         <v>55</v>
@@ -2423,7 +2423,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B11">
         <v>48</v>
@@ -2440,7 +2440,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B12">
         <v>85</v>
@@ -2457,7 +2457,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B13">
         <v>52</v>
@@ -2474,7 +2474,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B14">
         <v>50</v>
@@ -2491,7 +2491,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B15">
         <v>25.2</v>
@@ -2508,7 +2508,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B16">
         <v>66.5</v>
@@ -2525,7 +2525,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B17">
         <v>58</v>
@@ -2542,7 +2542,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B18">
         <v>158</v>
@@ -2559,7 +2559,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B19">
         <v>27</v>
@@ -2576,7 +2576,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B20">
         <v>123.7</v>
@@ -2593,7 +2593,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B21">
         <v>15</v>
@@ -2610,7 +2610,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B22">
         <v>17.96</v>
@@ -2627,7 +2627,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B23">
         <v>55.8</v>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B24">
         <v>87</v>
@@ -2661,7 +2661,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B25">
         <v>103.67</v>
@@ -2678,7 +2678,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B26">
         <v>129.13999999999999</v>
@@ -2695,7 +2695,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B27">
         <v>4.5199999999999996</v>
@@ -2712,7 +2712,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B28">
         <v>160.29</v>
@@ -2729,7 +2729,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B29">
         <v>62.2</v>
@@ -2746,7 +2746,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B30">
         <v>146.25</v>
@@ -2763,7 +2763,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B31">
         <v>48.35</v>
@@ -2780,7 +2780,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B32">
         <v>2.9</v>
@@ -2797,7 +2797,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B33">
         <v>12.3</v>
@@ -2833,7 +2833,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2841,16 +2841,16 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2864,10 +2864,10 @@
         <v>162</v>
       </c>
       <c r="D3" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2881,7 +2881,7 @@
         <v>162</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E4" s="31" t="s">
         <v>64</v>
@@ -2898,10 +2898,10 @@
         <v>161</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2915,7 +2915,7 @@
         <v>161</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>64</v>
@@ -2932,10 +2932,10 @@
         <v>163</v>
       </c>
       <c r="D7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2949,7 +2949,7 @@
         <v>163</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>64</v>
@@ -3010,49 +3010,49 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>359</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>360</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>361</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>362</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>364</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>8</v>
@@ -3075,7 +3075,7 @@
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -3087,22 +3087,22 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>371</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>373</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -3140,57 +3140,57 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="E2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="G2" s="6" t="s">
         <v>323</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>325</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="I2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="K2" t="s">
+        <v>325</v>
+      </c>
+      <c r="L2" t="s">
         <v>326</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>327</v>
       </c>
-      <c r="L2" t="s">
+      <c r="N2" t="s">
         <v>328</v>
-      </c>
-      <c r="M2" t="s">
-        <v>329</v>
-      </c>
-      <c r="N2" t="s">
-        <v>330</v>
       </c>
       <c r="O2" t="s">
         <v>102</v>
       </c>
       <c r="P2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="Q2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -3198,16 +3198,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E3" t="s">
         <v>270</v>
-      </c>
-      <c r="C3" t="s">
-        <v>331</v>
-      </c>
-      <c r="D3" t="s">
-        <v>283</v>
-      </c>
-      <c r="E3" t="s">
-        <v>272</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -3223,16 +3223,16 @@
         <v>4</v>
       </c>
       <c r="J3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="K3" t="s">
+        <v>330</v>
+      </c>
+      <c r="L3" t="s">
+        <v>331</v>
+      </c>
+      <c r="M3" t="s">
         <v>332</v>
-      </c>
-      <c r="L3" t="s">
-        <v>333</v>
-      </c>
-      <c r="M3" t="s">
-        <v>334</v>
       </c>
       <c r="N3" t="s">
         <v>128</v>
@@ -3241,10 +3241,10 @@
         <v>106</v>
       </c>
       <c r="P3" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="Q3" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -3252,22 +3252,22 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H4" t="s">
         <v>146</v>
@@ -3277,39 +3277,39 @@
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="K4" t="s">
         <v>103</v>
       </c>
       <c r="L4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="M4" t="s">
         <v>105</v>
       </c>
       <c r="O4" t="s">
+        <v>346</v>
+      </c>
+      <c r="P4" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q4" t="s">
         <v>348</v>
-      </c>
-      <c r="P4" t="s">
-        <v>349</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F5" t="s">
         <v>20</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="H5" t="s">
         <v>161</v>
@@ -3322,21 +3322,21 @@
         <v>105</v>
       </c>
       <c r="O5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="Q5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F6" t="s">
         <v>27</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H6" t="s">
         <v>162</v>
@@ -3346,15 +3346,15 @@
         <v>4</v>
       </c>
       <c r="O6" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="Q6" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F7" t="s">
         <v>30</v>
@@ -3367,10 +3367,10 @@
         <v>4</v>
       </c>
       <c r="O7" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="Q7" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -3435,7 +3435,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="H13" s="30" t="s">
         <v>169</v>
@@ -3447,7 +3447,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H14" s="30" t="s">
         <v>170</v>
@@ -3471,7 +3471,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="H16" s="30" t="s">
         <v>172</v>
@@ -3857,7 +3857,7 @@
         <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3877,19 +3877,19 @@
         <v>102</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>249</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>10</v>
@@ -3914,13 +3914,13 @@
         <v>106</v>
       </c>
       <c r="F3" t="s">
+        <v>376</v>
+      </c>
+      <c r="G3" t="s">
+        <v>377</v>
+      </c>
+      <c r="H3" t="s">
         <v>378</v>
-      </c>
-      <c r="G3" t="s">
-        <v>379</v>
-      </c>
-      <c r="H3" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -3940,10 +3940,10 @@
         <v>106</v>
       </c>
       <c r="G4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3967,13 +3967,13 @@
         <v>106</v>
       </c>
       <c r="F6" t="s">
+        <v>376</v>
+      </c>
+      <c r="G6" t="s">
+        <v>377</v>
+      </c>
+      <c r="H6" t="s">
         <v>378</v>
-      </c>
-      <c r="G6" t="s">
-        <v>379</v>
-      </c>
-      <c r="H6" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3993,10 +3993,10 @@
         <v>106</v>
       </c>
       <c r="G7" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I7" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -4020,13 +4020,13 @@
         <v>106</v>
       </c>
       <c r="F9" t="s">
+        <v>376</v>
+      </c>
+      <c r="G9" t="s">
+        <v>377</v>
+      </c>
+      <c r="H9" t="s">
         <v>378</v>
-      </c>
-      <c r="G9" t="s">
-        <v>379</v>
-      </c>
-      <c r="H9" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -4046,10 +4046,10 @@
         <v>106</v>
       </c>
       <c r="G10" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I10" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -4108,16 +4108,16 @@
         <v>106</v>
       </c>
       <c r="F17" t="s">
+        <v>376</v>
+      </c>
+      <c r="G17" t="s">
+        <v>377</v>
+      </c>
+      <c r="H17" t="s">
         <v>378</v>
       </c>
-      <c r="G17" t="s">
-        <v>379</v>
-      </c>
-      <c r="H17" t="s">
-        <v>380</v>
-      </c>
       <c r="K17" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -4137,10 +4137,10 @@
         <v>106</v>
       </c>
       <c r="G18" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I18" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -4238,7 +4238,7 @@
         <v>188</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>189</v>
@@ -4252,7 +4252,7 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D3" t="s">
         <v>191</v>
@@ -4386,7 +4386,7 @@
         <v>201</v>
       </c>
       <c r="C7" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D7" t="s">
         <v>196</v>
@@ -4421,7 +4421,7 @@
         <v>203</v>
       </c>
       <c r="C8" t="s">
-        <v>204</v>
+        <v>403</v>
       </c>
       <c r="D8" t="s">
         <v>196</v>
@@ -4439,7 +4439,7 @@
         <v>193</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L8" t="s">
         <v>194</v>
@@ -4450,10 +4450,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
+        <v>205</v>
+      </c>
+      <c r="C9" t="s">
         <v>206</v>
-      </c>
-      <c r="C9" t="s">
-        <v>207</v>
       </c>
       <c r="D9" t="s">
         <v>196</v>
@@ -4467,7 +4467,7 @@
         <v>193</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M9">
         <v>1</v>
@@ -4475,10 +4475,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D10" t="s">
         <v>196</v>
@@ -4492,7 +4492,7 @@
         <v>193</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M10">
         <v>1</v>
@@ -4500,13 +4500,13 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B11" t="s">
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D11" t="s">
         <v>196</v>
@@ -4535,13 +4535,13 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B12" t="s">
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D12" t="s">
         <v>196</v>
@@ -4559,10 +4559,10 @@
         <v>193</v>
       </c>
       <c r="K12" s="26" t="s">
+        <v>210</v>
+      </c>
+      <c r="L12" t="s">
         <v>211</v>
-      </c>
-      <c r="L12" t="s">
-        <v>212</v>
       </c>
       <c r="M12">
         <v>1</v>
@@ -4570,13 +4570,13 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B13" t="s">
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D13" t="s">
         <v>196</v>
@@ -4611,7 +4611,7 @@
         <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>214</v>
+        <v>404</v>
       </c>
       <c r="D14" t="s">
         <v>196</v>
@@ -4640,13 +4640,13 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B15" t="s">
         <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D15" t="s">
         <v>196</v>
@@ -4664,7 +4664,7 @@
         <v>193</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L15" t="s">
         <v>194</v>
@@ -4675,13 +4675,13 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B16" t="s">
         <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D16" t="s">
         <v>196</v>
@@ -4699,7 +4699,7 @@
         <v>193</v>
       </c>
       <c r="K16" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L16" t="s">
         <v>194</v>
@@ -4710,13 +4710,13 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B17" t="s">
         <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D17" t="s">
         <v>196</v>
@@ -4734,7 +4734,7 @@
         <v>193</v>
       </c>
       <c r="K17" s="36" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L17" t="s">
         <v>194</v>
@@ -4745,13 +4745,13 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B18" t="s">
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D18" t="s">
         <v>196</v>
@@ -4780,13 +4780,13 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B19" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C19" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D19" t="s">
         <v>196</v>
@@ -4815,13 +4815,13 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C20" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D20" t="s">
         <v>196</v>
@@ -4850,16 +4850,16 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>227</v>
+      </c>
+      <c r="B21" t="s">
+        <v>228</v>
+      </c>
+      <c r="C21" t="s">
+        <v>226</v>
+      </c>
+      <c r="D21" t="s">
         <v>229</v>
-      </c>
-      <c r="B21" t="s">
-        <v>230</v>
-      </c>
-      <c r="C21" t="s">
-        <v>228</v>
-      </c>
-      <c r="D21" t="s">
-        <v>231</v>
       </c>
       <c r="E21" t="s">
         <v>192</v>
@@ -4871,13 +4871,13 @@
         <v>5</v>
       </c>
       <c r="I21" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="J21" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="K21" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L21" t="s">
         <v>194</v>
@@ -4888,13 +4888,13 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B22" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C22" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D22" t="s">
         <v>196</v>
@@ -4917,16 +4917,16 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B23" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C23" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D23" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F23" s="3">
         <v>0</v>
@@ -4935,10 +4935,10 @@
         <v>0.5</v>
       </c>
       <c r="I23" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="J23" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="K23" s="21" t="s">
         <v>35</v>
@@ -4952,13 +4952,13 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>238</v>
+      </c>
+      <c r="B24" t="s">
+        <v>239</v>
+      </c>
+      <c r="C24" t="s">
         <v>240</v>
-      </c>
-      <c r="B24" t="s">
-        <v>241</v>
-      </c>
-      <c r="C24" t="s">
-        <v>242</v>
       </c>
       <c r="D24" t="s">
         <v>196</v>
@@ -4975,7 +4975,7 @@
         <v>37</v>
       </c>
       <c r="L24" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M24">
         <v>1</v>
@@ -4983,13 +4983,13 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C25" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D25" t="s">
         <v>196</v>
@@ -5007,10 +5007,10 @@
         <v>193</v>
       </c>
       <c r="K25" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L25" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M25">
         <v>2</v>
@@ -5033,12 +5033,12 @@
         <v>193</v>
       </c>
       <c r="K26" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
@@ -5053,10 +5053,10 @@
         <v>193</v>
       </c>
       <c r="K27" s="36" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L27" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M27">
         <v>1</v>
@@ -5064,7 +5064,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -5079,7 +5079,7 @@
         <v>193</v>
       </c>
       <c r="K28" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L28" t="s">
         <v>194</v>
@@ -5090,10 +5090,10 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B29" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C29" t="s">
         <v>17</v>
@@ -5119,10 +5119,10 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B30" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C30" t="s">
         <v>17</v>
@@ -5148,10 +5148,10 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C31" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D31" t="s">
         <v>196</v>
@@ -5160,10 +5160,10 @@
         <v>192</v>
       </c>
       <c r="I31" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="K31" s="36" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L31" t="s">
         <v>194</v>
@@ -6051,7 +6051,7 @@
         <v>28</v>
       </c>
       <c r="C27" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D27">
         <v>1585</v>
@@ -6060,7 +6060,7 @@
         <v>2158</v>
       </c>
       <c r="F27" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -6153,7 +6153,7 @@
         <v>28</v>
       </c>
       <c r="C33" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="D33">
         <v>2158</v>
@@ -6162,7 +6162,7 @@
         <v>2365</v>
       </c>
       <c r="F33" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
@@ -6378,7 +6378,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6386,13 +6386,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>157</v>
@@ -6429,7 +6429,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -6471,7 +6471,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -6485,7 +6485,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -6499,7 +6499,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -6541,7 +6541,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -6583,7 +6583,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -6597,7 +6597,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -6611,7 +6611,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="25" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -6633,13 +6633,13 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -6647,13 +6647,13 @@
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C23">
         <v>0</v>
       </c>
       <c r="F23" s="24" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -6692,67 +6692,67 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="D2" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="M2" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>266</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F3">
         <v>0.03</v>
@@ -6779,7 +6779,7 @@
         <v>0.6</v>
       </c>
       <c r="N3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -6787,7 +6787,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B4" s="3">
         <v>2.68</v>
@@ -6797,17 +6797,17 @@
         <v>1.0229999999999999</v>
       </c>
       <c r="E4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F5">
         <v>0.03</v>
@@ -6834,7 +6834,7 @@
         <v>0.6</v>
       </c>
       <c r="N5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -6842,12 +6842,12 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="E6" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="H6">
         <v>1.0699999999999999E-2</v>
@@ -6893,10 +6893,10 @@
         <v>0</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6904,25 +6904,25 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>279</v>
-      </c>
       <c r="H2" s="8" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6933,10 +6933,10 @@
       <c r="C3" s="31"/>
       <c r="D3" s="31"/>
       <c r="E3" s="31" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
@@ -6946,7 +6946,7 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -6955,16 +6955,16 @@
         <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H4" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6972,7 +6972,7 @@
         <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -6981,16 +6981,16 @@
         <v>162</v>
       </c>
       <c r="E5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G5" t="s">
         <v>87</v>
       </c>
       <c r="H5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6998,7 +6998,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>28</v>
@@ -7007,16 +7007,16 @@
         <v>162</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G6" s="31">
         <v>1</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -7024,7 +7024,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -7033,16 +7033,16 @@
         <v>162</v>
       </c>
       <c r="E7" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="G7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H7" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -7050,7 +7050,7 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -7059,16 +7059,16 @@
         <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="F8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7076,7 +7076,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>28</v>
@@ -7085,16 +7085,16 @@
         <v>162</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G9" s="31">
         <v>1</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -7102,7 +7102,7 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C10" t="s">
         <v>28</v>
@@ -7111,16 +7111,16 @@
         <v>161</v>
       </c>
       <c r="E10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="F10" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G10">
         <v>0.9</v>
       </c>
       <c r="H10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -7128,7 +7128,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C11" t="s">
         <v>28</v>
@@ -7137,16 +7137,16 @@
         <v>161</v>
       </c>
       <c r="E11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F11" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G11" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H11" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7154,7 +7154,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>28</v>
@@ -7163,16 +7163,16 @@
         <v>161</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G12" s="31">
         <v>1</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -7180,7 +7180,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C13" t="s">
         <v>28</v>
@@ -7189,16 +7189,16 @@
         <v>163</v>
       </c>
       <c r="E13" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G13" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H13" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -7206,7 +7206,7 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C14" t="s">
         <v>28</v>
@@ -7215,16 +7215,16 @@
         <v>163</v>
       </c>
       <c r="E14" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F14" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G14" t="s">
         <v>87</v>
       </c>
       <c r="H14" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7232,7 +7232,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C15" s="31" t="s">
         <v>28</v>
@@ -7241,16 +7241,16 @@
         <v>163</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G15" s="31">
         <v>1</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -7258,7 +7258,7 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C16" t="s">
         <v>28</v>
@@ -7267,16 +7267,16 @@
         <v>163</v>
       </c>
       <c r="E16" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F16" t="s">
+        <v>395</v>
+      </c>
+      <c r="G16" t="s">
+        <v>280</v>
+      </c>
+      <c r="H16" t="s">
         <v>397</v>
-      </c>
-      <c r="G16" t="s">
-        <v>282</v>
-      </c>
-      <c r="H16" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -7284,7 +7284,7 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C17" t="s">
         <v>28</v>
@@ -7293,16 +7293,16 @@
         <v>163</v>
       </c>
       <c r="E17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G17" t="s">
         <v>87</v>
       </c>
       <c r="H17" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7310,7 +7310,7 @@
         <v>11</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C18" s="31" t="s">
         <v>28</v>
@@ -7319,21 +7319,21 @@
         <v>163</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F18" s="31" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G18" s="31">
         <v>1</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Detected a problem with how Project is reading wells from the project_table.xlsx
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_geo_py\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9026C1CA-D41D-4D58-890B-D64555C54D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670A4988-CD19-4DFC-B364-BA58BE42105A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7170" yWindow="3090" windowWidth="28800" windowHeight="15345" tabRatio="685" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-31905" yWindow="2910" windowWidth="28800" windowHeight="15345" tabRatio="685" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -3589,7 +3589,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>59</v>
@@ -3756,7 +3756,7 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>89</v>

</xml_diff>

<commit_message>
Remove calc_stats.py and its tests
calc_stat_class only used save_rokdoc_output() from the old calc_stats.py.
Move it to calc_stat_class.py as write_rokdoc_sums_and_averages(), and add a
test for it. The rest of calc_stats.py was unused, so delete it together
with test_calc_stats.py.

Remove seaborn and bruges from requirements.txt. seaborn was only used by
calc_stats.py, and the bruges code in use is the copy in
core/wavelets_from_bruges.py. Also commit the current project_table.xlsx,
and tick off the item in ToDo.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_geo_py\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_geo_py\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670A4988-CD19-4DFC-B364-BA58BE42105A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071BDF32-FA61-472A-966D-A4CE65479470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31905" yWindow="2910" windowWidth="28800" windowHeight="15345" tabRatio="685" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="930" windowWidth="32655" windowHeight="16785" tabRatio="685" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -3635,7 +3635,7 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>69</v>
@@ -3661,7 +3661,7 @@
         <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>73</v>
@@ -3687,7 +3687,7 @@
         <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>74</v>
@@ -3716,7 +3716,7 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>81</v>
@@ -3733,7 +3733,7 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>84</v>
@@ -3756,7 +3756,7 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>89</v>
@@ -3788,7 +3788,7 @@
         <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>91</v>

</xml_diff>

<commit_message>
Update the project table and the plot settings comment
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_geo_py\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071BDF32-FA61-472A-966D-A4CE65479470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F8A5D5-0309-437D-8A39-E41C1CF5DF28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="930" windowWidth="32655" windowHeight="16785" tabRatio="685" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="930" windowWidth="32655" windowHeight="16785" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -2077,7 +2077,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>12</v>
@@ -2097,7 +2097,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>15</v>

</xml_diff>